<commit_message>
tareas y consultas  parece ok
</commit_message>
<xml_diff>
--- a/plantillas_migracion/datos_cliente.xlsx
+++ b/plantillas_migracion/datos_cliente.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId3"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="123">
   <si>
     <t xml:space="preserve">razonSocial*</t>
   </si>
@@ -216,6 +216,9 @@
     <t xml:space="preserve">René Llivicura</t>
   </si>
   <si>
+    <t xml:space="preserve">0102345680</t>
+  </si>
+  <si>
     <t xml:space="preserve">croenlio merchan</t>
   </si>
   <si>
@@ -246,7 +249,7 @@
     <t xml:space="preserve">Piedad Orellana </t>
   </si>
   <si>
-    <t xml:space="preserve">piedad@mail.como</t>
+    <t xml:space="preserve">piedad@mail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Asistente</t>
@@ -343,6 +346,18 @@
   </si>
   <si>
     <t xml:space="preserve">notas_acuerdo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21-10-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">actor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mensual</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUCCIONES - datos_cliente.xlsx (lo llena EL CLIENTE)</t>
@@ -395,7 +410,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,12 +432,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u val="single"/>
@@ -496,7 +505,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -828,83 +837,83 @@
         <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>44</v>
       </c>
     </row>
@@ -930,68 +939,102 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.46"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="A2" s="4" t="n">
+        <v>123456</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H3" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1014,72 +1057,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1155,7 +1198,7 @@
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1413,14 +1456,14 @@
       <c r="B3" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>104649842</v>
+      <c r="C3" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>987414141</v>
@@ -1442,7 +1485,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1450,7 +1493,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>51</v>
@@ -1459,29 +1502,29 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>102455080</v>
@@ -1490,11 +1533,12 @@
         <v>987414244</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>72</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="F3" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
validaciones, errores 500, permisos y creaciones de juicios por perfiles ok
</commit_message>
<xml_diff>
--- a/plantillas_migracion/datos_cliente.xlsx
+++ b/plantillas_migracion/datos_cliente.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="119">
   <si>
     <t xml:space="preserve">razonSocial*</t>
   </si>
@@ -346,18 +346,6 @@
   </si>
   <si>
     <t xml:space="preserve">notas_acuerdo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21-10-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">actor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mensual</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUCCIONES - datos_cliente.xlsx (lo llena EL CLIENTE)</t>
@@ -484,7 +472,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -502,10 +490,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -994,47 +978,19 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
-        <v>123456</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>107</v>
-      </c>
+      <c r="A2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H3" s="5"/>
+      <c r="H3" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1057,72 +1013,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>